<commit_message>
Rename UndervoltageTemperatureAndCurrentFlagsInformation; update BMS CAN protocol docs
</commit_message>
<xml_diff>
--- a/docs/_static/Gen13 Battery Management System CAN Communication Protocol.xlsx
+++ b/docs/_static/Gen13 Battery Management System CAN Communication Protocol.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="87">
   <si>
     <t>Type</t>
   </si>
@@ -233,7 +233,7 @@
     <t>Undervoltage/temperature flags</t>
   </si>
   <si>
-    <t xml:space="preserve">[0-35: Cell 0.0, 0.1, ..., 5.5 undervoltage flags][36-53: Thermistor 0.0, 0.1, ..., 5.2 undertemperature flags][54-63: reserved]        </t>
+    <t xml:space="preserve">[0-35: Cell 0.0, 0.1, ..., 5.5 undervoltage flags][36-53: Thermistor 0.0, 0.1, ..., 5.2 undertemperature flags][54: undercurrent flag][55-63: reserved]        </t>
   </si>
   <si>
     <t>Low Voltage Bus voltage and current</t>
@@ -269,7 +269,10 @@
     <t>[0: horn status][1-63: reserved]</t>
   </si>
   <si>
-    <t>5-31</t>
+    <t>5-30</t>
+  </si>
+  <si>
+    <t>Heartbeat</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,8 @@
     <col customWidth="1" min="2" max="2" width="9.5"/>
     <col customWidth="1" min="3" max="3" width="19.0"/>
     <col customWidth="1" min="4" max="4" width="20.75"/>
-    <col customWidth="1" min="5" max="6" width="52.25"/>
+    <col customWidth="1" min="5" max="5" width="52.25"/>
+    <col customWidth="1" min="6" max="6" width="54.5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1176,6 +1180,20 @@
         <v>79</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="7">
+        <v>31.0</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="E8:F8"/>
@@ -1187,7 +1205,7 @@
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="B3:B8"/>
-    <mergeCell ref="C3:C8"/>
+    <mergeCell ref="C3:C9"/>
     <mergeCell ref="E3:F6"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>

</xml_diff>

<commit_message>
Moved battery flag hold logic onto phub
</commit_message>
<xml_diff>
--- a/docs/_static/Gen13 Battery Management System CAN Communication Protocol.xlsx
+++ b/docs/_static/Gen13 Battery Management System CAN Communication Protocol.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="86">
   <si>
     <t>Type</t>
   </si>
@@ -218,7 +218,7 @@
     <t>Statuses</t>
   </si>
   <si>
-    <t>[0: relay status][1: electric safe discharge status][2: discharge status][3-31: reserved]</t>
+    <t>[0: relay status][1: electric safe discharge status][2: discharge status][3-23: reserved][24-31: flag_hold]</t>
   </si>
   <si>
     <t>Supplementary battery voltage (float)</t>
@@ -269,10 +269,7 @@
     <t>[0: horn status][1-63: reserved]</t>
   </si>
   <si>
-    <t>5-30</t>
-  </si>
-  <si>
-    <t>Heartbeat</t>
+    <t>5-31</t>
   </si>
 </sst>
 </file>
@@ -1137,6 +1134,7 @@
       <c r="A4" s="6" t="s">
         <v>80</v>
       </c>
+      <c r="C4" s="7"/>
       <c r="D4" s="7">
         <v>1.0</v>
       </c>
@@ -1145,6 +1143,7 @@
       <c r="A5" s="6" t="s">
         <v>81</v>
       </c>
+      <c r="C5" s="7"/>
       <c r="D5" s="7">
         <v>2.0</v>
       </c>
@@ -1153,6 +1152,7 @@
       <c r="A6" s="6" t="s">
         <v>82</v>
       </c>
+      <c r="C6" s="7"/>
       <c r="D6" s="7">
         <v>3.0</v>
       </c>
@@ -1161,6 +1161,7 @@
       <c r="A7" s="6" t="s">
         <v>83</v>
       </c>
+      <c r="C7" s="7"/>
       <c r="D7" s="7">
         <v>4.0</v>
       </c>
@@ -1173,6 +1174,7 @@
       <c r="A8" s="6" t="s">
         <v>79</v>
       </c>
+      <c r="C8" s="7"/>
       <c r="D8" s="9" t="s">
         <v>85</v>
       </c>
@@ -1181,21 +1183,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" s="7">
-        <v>0.1</v>
-      </c>
-      <c r="D9" s="7">
-        <v>31.0</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>79</v>
-      </c>
+      <c r="A9" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E33:F33"/>
@@ -1205,7 +1196,6 @@
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="B3:B8"/>
-    <mergeCell ref="C3:C9"/>
     <mergeCell ref="E3:F6"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>

</xml_diff>